<commit_message>
Replace project with updated InfraESG analytics
</commit_message>
<xml_diff>
--- a/data/InfraESG_Report.xlsx
+++ b/data/InfraESG_Report.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -504,7 +504,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Portfolio Carbon Intensity (tCO₂e/€M)</t>
+          <t>Avg Carbon Intensity (tCO₂e/€M rev)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -538,6 +538,16 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SFDR Data Gaps (disclosed)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>3</v>
       </c>
     </row>
@@ -566,7 +576,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -656,7 +666,7 @@
         <v>82</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>45.93023255813954</v>
+        <v>45.9</v>
       </c>
       <c r="J2" s="4" t="n">
         <v>91</v>
@@ -696,7 +706,7 @@
         <v>80</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>8.246753246753247</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J3" s="4" t="n">
         <v>78</v>
@@ -736,7 +746,7 @@
         <v>78</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>33.95061728395061</v>
+        <v>34</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>95</v>
@@ -776,7 +786,7 @@
         <v>80</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>114.8148148148148</v>
+        <v>114.8</v>
       </c>
       <c r="J5" s="4" t="n">
         <v>35</v>
@@ -816,7 +826,7 @@
         <v>75</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>888.9679715302491</v>
+        <v>889</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>65</v>
@@ -856,7 +866,7 @@
         <v>76</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>187.1951219512195</v>
+        <v>187.2</v>
       </c>
       <c r="J7" s="4" t="n">
         <v>96</v>
@@ -896,7 +906,7 @@
         <v>75</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>267.6767676767677</v>
+        <v>267.7</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>42</v>
@@ -936,7 +946,7 @@
         <v>73</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>338.5454545454546</v>
+        <v>338.5</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>75</v>
@@ -976,7 +986,7 @@
         <v>70</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>124.2857142857143</v>
+        <v>124.3</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>40</v>
@@ -1016,7 +1026,7 @@
         <v>75</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>937.2549019607843</v>
+        <v>937.3</v>
       </c>
       <c r="J11" s="4" t="n">
         <v>22</v>
@@ -1056,7 +1066,7 @@
         <v>72</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>116.1764705882353</v>
+        <v>116.2</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>15</v>
@@ -1096,7 +1106,7 @@
         <v>72</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>101.8018018018018</v>
+        <v>101.8</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>42</v>
@@ -1136,7 +1146,7 @@
         <v>74</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>284.5794392523365</v>
+        <v>284.6</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>55</v>
@@ -1176,7 +1186,7 @@
         <v>70</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>2560.629921259843</v>
+        <v>2560.6</v>
       </c>
       <c r="J15" s="4" t="n">
         <v>38</v>
@@ -1216,7 +1226,7 @@
         <v>70</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>47.79411764705882</v>
+        <v>47.8</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>30</v>
@@ -1256,7 +1266,7 @@
         <v>72</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>122.5806451612903</v>
+        <v>122.6</v>
       </c>
       <c r="J17" s="4" t="n">
         <v>12</v>
@@ -1296,7 +1306,7 @@
         <v>72</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>1896.907216494845</v>
+        <v>1896.9</v>
       </c>
       <c r="J18" s="4" t="n">
         <v>18</v>
@@ -1336,7 +1346,7 @@
         <v>65</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>10.04366812227074</v>
+        <v>10</v>
       </c>
       <c r="J19" s="4" t="n">
         <v>55</v>
@@ -1376,7 +1386,7 @@
         <v>62</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>11.0738255033557</v>
+        <v>11.1</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>35</v>
@@ -1416,7 +1426,7 @@
         <v>68</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>1989.583333333333</v>
+        <v>1989.6</v>
       </c>
       <c r="J21" s="4" t="n">
         <v>22</v>
@@ -1456,7 +1466,7 @@
         <v>70</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>1999.183673469388</v>
+        <v>1999.2</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>15</v>
@@ -1496,7 +1506,7 @@
         <v>65</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>192.9583904892547</v>
+        <v>193</v>
       </c>
       <c r="J23" s="4" t="n">
         <v>8</v>
@@ -1536,7 +1546,7 @@
         <v>62</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>191.2136536030341</v>
+        <v>191.2</v>
       </c>
       <c r="J24" s="4" t="n">
         <v>5</v>
@@ -1576,7 +1586,7 @@
         <v>60</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>201.7232640648758</v>
+        <v>201.7</v>
       </c>
       <c r="J25" s="4" t="n">
         <v>6</v>
@@ -1616,7 +1626,7 @@
         <v>52</v>
       </c>
       <c r="I26" s="4" t="n">
-        <v>89.88764044943819</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="J26" s="4" t="n">
         <v>45</v>
@@ -1639,8 +1649,8 @@
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1687,15 +1697,15 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Scope 1+2+3 (weighted, kt CO₂e)</t>
+          <t>Financed Scope 1+2+3 emissions</t>
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>266047.6</v>
+        <v>1742792</v>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>kt CO₂e</t>
+          <t>tCO₂e</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -1715,11 +1725,11 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>tCO₂e per €M invested</t>
+          <t>Financed emissions per €M invested</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>17313.8</v>
+        <v>1742.8</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
@@ -1728,7 +1738,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1743,11 +1753,11 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>tCO₂e per €M revenue (weighted)</t>
+          <t>Weighted-avg GHG intensity (Scope 1+2+3)</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>547.6</v>
+        <v>1698.5</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
@@ -1756,7 +1766,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1781,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>% portfolio in fossil fuels</t>
+          <t>% portfolio in fossil fuel companies</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
@@ -1799,7 +1809,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Non-renewable energy share</t>
+          <t>Weighted non-renewable energy share</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
@@ -1827,20 +1837,20 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Energy consumption intensity</t>
+          <t>Energy intensity (proxy from Scope 2 / grid factor)</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>547.5700000000001</v>
+        <v>136</v>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>GWh / €M rev</t>
+          <t>MWh / €M rev</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1855,20 +1865,22 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Companies with biodiversity impact</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>0</v>
+          <t>Issuer-level biodiversity data not yet collected</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>n/a — data gap</t>
+        </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1883,20 +1895,22 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Tonnes of emissions to water</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>0</v>
+          <t>Issuer-level water emissions data not yet collected</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>n/a — data gap</t>
+        </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>tonnes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1911,20 +1925,22 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Hazardous waste ratio</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>0</v>
+          <t>Issuer-level hazardous waste data not yet collected</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>n/a — data gap</t>
+        </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>tonnes / €M rev</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1955,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Companies with UNGC violations</t>
+          <t>Companies with severe controversies (UNGC proxy)</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
@@ -1967,7 +1983,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Companies lacking compliance mechanisms</t>
+          <t>Companies with elevated controversy / weak processes</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
@@ -1995,20 +2011,20 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Management gender gap (proxy)</t>
+          <t>Gap to management gender parity (proxy for pay gap)</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>72.09999999999999</v>
+        <v>22.1</v>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>pp below 50%</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2067,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Exposure to controversial weapons</t>
+          <t>Exposure to controversial weapons (screened)</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
@@ -2864,7 +2880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2874,7 +2890,8 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2915,6 +2932,11 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
           <t>reduction_pct</t>
         </is>
       </c>
@@ -2948,7 +2970,10 @@
         <v>790</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>34.2</v>
+        <v>742</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>38.2</v>
       </c>
     </row>
     <row r="3">
@@ -2980,18 +3005,21 @@
         <v>6090</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>25.7</v>
+        <v>5710</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>30.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>ENPH</t>
+          <t>VWDRY</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Enphase Energy</t>
+          <t>Vestas Wind Systems</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -3000,30 +3028,33 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>30</v>
+        <v>165</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>26</v>
+        <v>148</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>24</v>
+        <v>135</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>23</v>
+        <v>127</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>23.3</v>
+        <v>120</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>27.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>VWDRY</t>
+          <t>ENPH</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Vestas Wind Systems</t>
+          <t>Enphase Energy</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -3032,19 +3063,22 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>165</v>
+        <v>30</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>148</v>
+        <v>26</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>135</v>
+        <v>24</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>127</v>
+        <v>23</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>26.7</v>
       </c>
     </row>
     <row r="6">
@@ -3076,7 +3110,10 @@
         <v>165</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>21.4</v>
+        <v>158</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>24.8</v>
       </c>
     </row>
     <row r="7">
@@ -3108,7 +3145,10 @@
         <v>2480</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>20</v>
+        <v>2360</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>23.9</v>
       </c>
     </row>
     <row r="8">
@@ -3140,71 +3180,80 @@
         <v>1535</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>19.2</v>
+        <v>1472</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>22.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>WELL</t>
+          <t>AES</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Welltower</t>
+          <t>AES Corporation</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Social Infrastructure</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>950</v>
+        <v>38000</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>880</v>
+        <v>36500</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>820</v>
+        <v>34500</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>790</v>
+        <v>32520</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>16.8</v>
+        <v>30200</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>20.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>FSLR</t>
+          <t>WELL</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>First Solar</t>
+          <t>Welltower</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Renewable Energy</t>
+          <t>Social Infrastructure</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>520</v>
+        <v>950</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>480</v>
+        <v>880</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>450</v>
+        <v>820</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>435</v>
+        <v>790</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>16.3</v>
+        <v>762</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>19.8</v>
       </c>
     </row>
     <row r="11">
@@ -3236,71 +3285,80 @@
         <v>1130</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>16.3</v>
+        <v>1086</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>19.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>FSLR</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Digital Realty</t>
+          <t>First Solar</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Digital Infrastructure</t>
+          <t>Renewable Energy</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>2200</v>
+        <v>520</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>2050</v>
+        <v>480</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>1920</v>
+        <v>450</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>1862</v>
+        <v>435</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>15.4</v>
+        <v>421</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>BIP</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Brookfield Infrastructure</t>
+          <t>Digital Realty</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Digital Infrastructure</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>6200</v>
+        <v>2200</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>5800</v>
+        <v>2050</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>5500</v>
+        <v>1920</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>5300</v>
+        <v>1862</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>14.5</v>
+        <v>1801</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>18.1</v>
       </c>
     </row>
     <row r="14">
@@ -3332,39 +3390,45 @@
         <v>325</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>14.5</v>
+        <v>312</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>17.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>AES</t>
+          <t>BIP</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>AES Corporation</t>
+          <t>Brookfield Infrastructure</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>38000</v>
+        <v>6200</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>36500</v>
+        <v>5800</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>34500</v>
+        <v>5500</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>32520</v>
+        <v>5300</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14.4</v>
+        <v>5110</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>17.6</v>
       </c>
     </row>
     <row r="16">
@@ -3396,71 +3460,80 @@
         <v>28650</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>13.2</v>
+        <v>27500</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>16.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>SEDG</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>SolarEdge Technologies</t>
+          <t>Southern Company</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Renewable Energy</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>38</v>
+        <v>56000</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>36</v>
+        <v>54000</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>34</v>
+        <v>51500</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>33</v>
+        <v>48980</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>13.2</v>
+        <v>46900</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>16.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>SEDG</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Southern Company</t>
+          <t>SolarEdge Technologies</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Renewable Energy</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>56000</v>
+        <v>38</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>54000</v>
+        <v>36</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>51500</v>
+        <v>34</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>48980</v>
+        <v>33</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>12.5</v>
+        <v>32</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>15.8</v>
       </c>
     </row>
     <row r="19">
@@ -3492,7 +3565,10 @@
         <v>24980</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>11.4</v>
+        <v>23950</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>15.1</v>
       </c>
     </row>
     <row r="20">
@@ -3524,7 +3600,10 @@
         <v>55200</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>11</v>
+        <v>53100</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>14.4</v>
       </c>
     </row>
     <row r="21">
@@ -3556,7 +3635,10 @@
         <v>60500</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>11</v>
+        <v>58950</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>13.3</v>
       </c>
     </row>
     <row r="22">
@@ -3588,7 +3670,10 @@
         <v>12920</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>10.9</v>
+        <v>12610</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="23">
@@ -3620,7 +3705,10 @@
         <v>39800</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>9.5</v>
+        <v>38700</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="24">
@@ -3652,7 +3740,10 @@
         <v>19120</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>9</v>
+        <v>18700</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="25">
@@ -3684,7 +3775,10 @@
         <v>42200</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>6.2</v>
+        <v>41350</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>8.1</v>
       </c>
     </row>
     <row r="26">
@@ -3716,7 +3810,10 @@
         <v>80</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-11.1</v>
+        <v>82</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>-13.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>